<commit_message>
Document and verify the v6 boss move effects P0 rollout
Record 19 active representatives, normalized effects, legacy v5 replay and actual X11 checks; keep remaining119 explicit and EXE generation on hold.
</commit_message>
<xml_diff>
--- a/docs/boss-ace-tactics.xlsx
+++ b/docs/boss-ace-tactics.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구현 순서" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'대표 전술안'!$A$1:$M$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'대표 전술안'!$A$1:$N$139</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'기술 효과'!$A$1:$I$234</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'구현 순서'!$A$1:$C$14</definedName>
   </definedNames>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M139"/>
+  <dimension ref="A1:N139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -448,6 +448,7 @@
     <col width="70" customWidth="1" min="11" max="11"/>
     <col width="70" customWidth="1" min="12" max="12"/>
     <col width="80" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -516,6 +517,11 @@
           <t>출처</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>적용 현황</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -583,6 +589,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -650,6 +661,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -717,6 +733,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -784,6 +805,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/gymrematch.shtml</t>
         </is>
       </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -851,6 +877,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/gymrematch.shtml</t>
         </is>
       </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -918,6 +949,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -985,6 +1021,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/gymrematch.shtml</t>
         </is>
       </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1052,6 +1093,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/gyms.shtml</t>
         </is>
       </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1119,6 +1165,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1186,6 +1237,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1253,6 +1309,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1320,6 +1381,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1387,6 +1453,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1454,6 +1525,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1521,6 +1597,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1588,6 +1669,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1655,6 +1741,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1722,6 +1813,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1789,6 +1885,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1856,6 +1957,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1923,6 +2029,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1990,6 +2101,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2057,6 +2173,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2124,6 +2245,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2191,6 +2317,11 @@
           <t>https://github.com/pret/pokeemerald/blob/731ad5bfd6e6f265508d0efcca0ba42f9dcf5881/src/data/trainer_parties.h</t>
         </is>
       </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2258,6 +2389,11 @@
           <t>https://github.com/pret/pokeemerald/blob/731ad5bfd6e6f265508d0efcca0ba42f9dcf5881/src/data/trainer_parties.h</t>
         </is>
       </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2325,6 +2461,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/gyms.shtml</t>
         </is>
       </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2392,6 +2533,11 @@
           <t>https://github.com/pret/pokeemerald/blob/731ad5bfd6e6f265508d0efcca0ba42f9dcf5881/src/data/trainer_parties.h</t>
         </is>
       </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2459,6 +2605,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_roark_rematch.json</t>
         </is>
       </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2526,6 +2677,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_gardenia_rematch.json</t>
         </is>
       </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2593,6 +2749,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_maylene_rematch.json</t>
         </is>
       </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2660,6 +2821,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_wake_rematch.json</t>
         </is>
       </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2727,6 +2893,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_fantina_rematch.json</t>
         </is>
       </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2794,6 +2965,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_byron_rematch.json</t>
         </is>
       </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2861,6 +3037,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_candice_rematch.json</t>
         </is>
       </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2928,6 +3109,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/leader_volkner_rematch.json</t>
         </is>
       </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2995,6 +3181,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3062,6 +3253,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3129,6 +3325,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3196,6 +3397,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3263,6 +3469,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3330,6 +3541,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3397,6 +3613,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3464,6 +3685,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3531,6 +3757,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3598,6 +3829,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3665,6 +3901,11 @@
           <t>https://www.serebii.net/blackwhite/gyms.shtml</t>
         </is>
       </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3732,6 +3973,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3799,6 +4045,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3866,6 +4117,11 @@
           <t>https://www.serebii.net/black2white2/gyms.shtml</t>
         </is>
       </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3933,6 +4189,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4000,6 +4261,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4067,6 +4333,11 @@
           <t>https://bulbapedia.bulbagarden.net/wiki/Tower_of_Mastery</t>
         </is>
       </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4134,6 +4405,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4201,6 +4477,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4268,6 +4549,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4335,6 +4621,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -4402,6 +4693,11 @@
           <t>https://www.serebii.net/xy/gyms.shtml</t>
         </is>
       </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4469,6 +4765,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4536,6 +4837,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4603,6 +4909,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -4670,6 +4981,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4737,6 +5053,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4804,6 +5125,11 @@
           <t>https://www.serebii.net/swordshield/gyms.shtml</t>
         </is>
       </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4871,6 +5197,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4938,6 +5269,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5005,6 +5341,11 @@
           <t>https://www.serebii.net/swordshield/gyms.shtml</t>
         </is>
       </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5072,6 +5413,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5139,6 +5485,11 @@
           <t>https://www.serebii.net/swordshield/championcuprematch.shtml</t>
         </is>
       </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5206,6 +5557,11 @@
           <t>https://www.serebii.net/swordshield/marnie.shtml</t>
         </is>
       </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5273,6 +5629,11 @@
           <t>https://www.serebii.net/swordshield/klaraavery.shtml</t>
         </is>
       </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5340,6 +5701,11 @@
           <t>https://www.serebii.net/swordshield/klaraavery.shtml</t>
         </is>
       </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5407,6 +5773,11 @@
           <t>https://www.serebii.net/swordshield/mustard.shtml</t>
         </is>
       </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -5474,6 +5845,11 @@
           <t>https://www.serebii.net/swordshield/dailyevent.shtml</t>
         </is>
       </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5541,6 +5917,11 @@
           <t>https://www.serebii.net/scarletviolet/academyacetournament.shtml</t>
         </is>
       </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5608,6 +5989,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5675,6 +6061,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -5742,6 +6133,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -5809,6 +6205,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5876,6 +6277,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5943,6 +6349,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -6010,6 +6421,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -6077,6 +6493,11 @@
           <t>https://www.serebii.net/scarletviolet/gymrematches.shtml</t>
         </is>
       </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -6144,6 +6565,11 @@
           <t>https://www.serebii.net/sunmoon/grandtrials.shtml</t>
         </is>
       </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6211,6 +6637,11 @@
           <t>https://www.serebii.net/sunmoon/grandtrials.shtml</t>
         </is>
       </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6278,6 +6709,11 @@
           <t>https://www.serebii.net/sunmoon/grandtrials.shtml</t>
         </is>
       </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -6345,6 +6781,11 @@
           <t>https://www.serebii.net/ultrasunultramoon/grandtrials.shtml</t>
         </is>
       </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6412,6 +6853,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -6479,6 +6925,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -6546,6 +6997,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6613,6 +7069,11 @@
           <t>https://www.serebii.net/letsgopikachueevee/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6680,6 +7141,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6747,6 +7213,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6814,6 +7285,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -6881,6 +7357,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -6948,6 +7429,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7015,6 +7501,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7082,6 +7573,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -7149,6 +7645,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/elite_four_aaron.json</t>
         </is>
       </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7216,6 +7717,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/elite_four_bertha.json</t>
         </is>
       </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7283,6 +7789,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/elite_four_flint.json</t>
         </is>
       </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -7350,6 +7861,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/elite_four_lucian.json</t>
         </is>
       </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -7417,6 +7933,11 @@
           <t>https://www.serebii.net/black2white2/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7484,6 +8005,11 @@
           <t>https://www.serebii.net/black2white2/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -7551,6 +8077,11 @@
           <t>https://www.serebii.net/black2white2/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7618,6 +8149,11 @@
           <t>https://www.serebii.net/black2white2/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7685,6 +8221,11 @@
           <t>https://www.serebii.net/xy/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7752,6 +8293,11 @@
           <t>https://www.serebii.net/xy/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7819,6 +8365,11 @@
           <t>https://www.serebii.net/xy/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7886,6 +8437,11 @@
           <t>https://www.serebii.net/xy/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -7953,6 +8509,11 @@
           <t>https://www.serebii.net/sunmoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8020,6 +8581,11 @@
           <t>https://www.serebii.net/sunmoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8087,6 +8653,11 @@
           <t>https://www.serebii.net/sunmoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8154,6 +8725,11 @@
           <t>https://www.serebii.net/sunmoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8221,6 +8797,11 @@
           <t>https://www.serebii.net/scarletviolet/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8288,6 +8869,11 @@
           <t>https://www.serebii.net/scarletviolet/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8355,6 +8941,11 @@
           <t>https://www.serebii.net/scarletviolet/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8422,6 +9013,11 @@
           <t>https://www.serebii.net/scarletviolet/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8489,6 +9085,11 @@
           <t>https://www.serebii.net/ultrasunultramoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -8556,6 +9157,11 @@
           <t>https://www.serebii.net/scarletviolet/blueberryelitefour.shtml</t>
         </is>
       </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -8623,6 +9229,11 @@
           <t>https://www.serebii.net/scarletviolet/blueberryelitefour.shtml</t>
         </is>
       </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8690,6 +9301,11 @@
           <t>https://www.serebii.net/scarletviolet/blueberryelitefour.shtml</t>
         </is>
       </c>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -8757,6 +9373,11 @@
           <t>https://www.serebii.net/scarletviolet/blueberryelitefour.shtml</t>
         </is>
       </c>
+      <c r="N124" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8824,6 +9445,11 @@
           <t>https://www.serebii.net/rb/rival.shtml</t>
         </is>
       </c>
+      <c r="N125" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -8891,6 +9517,11 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N126" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -8958,6 +9589,11 @@
           <t>https://www.serebii.net/omegarubyalphasapphire/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N127" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9025,6 +9661,11 @@
           <t>https://github.com/pret/pokeemerald/blob/731ad5bfd6e6f265508d0efcca0ba42f9dcf5881/src/data/trainer_parties.h</t>
         </is>
       </c>
+      <c r="N128" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9092,6 +9733,11 @@
           <t>https://github.com/pret/pokeplatinum/blob/1dc13dcea40c04ab53f1f607de46023dc409ef20/res/trainers/data/champion_cynthia.json</t>
         </is>
       </c>
+      <c r="N129" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -9159,6 +9805,11 @@
           <t>https://www.serebii.net/blackwhite/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N130" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -9226,6 +9877,11 @@
           <t>https://www.serebii.net/black2white2/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N131" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -9293,6 +9949,11 @@
           <t>https://www.serebii.net/xy/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N132" s="2" t="inlineStr">
+        <is>
+          <t>v6 P0 적용</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -9360,6 +10021,11 @@
           <t>https://www.serebii.net/swordshield/championcup.shtml</t>
         </is>
       </c>
+      <c r="N133" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -9427,6 +10093,11 @@
           <t>https://www.serebii.net/scarletviolet/academyacetournament.shtml</t>
         </is>
       </c>
+      <c r="N134" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -9494,6 +10165,11 @@
           <t>https://www.serebii.net/scarletviolet/victoryroad.shtml</t>
         </is>
       </c>
+      <c r="N135" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -9561,6 +10237,11 @@
           <t>https://www.serebii.net/sunmoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N136" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -9628,6 +10309,11 @@
           <t>https://www.serebii.net/ultrasunultramoon/elitefour.shtml</t>
         </is>
       </c>
+      <c r="N137" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9695,6 +10381,11 @@
           <t>https://www.serebii.net/scarletviolet/blueberryelitefour.shtml</t>
         </is>
       </c>
+      <c r="N138" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -9762,9 +10453,14 @@
           <t>https://github.com/pret/pokeheartgold/blob/75912a082f196496b4f9d347e0f99319150a96b4/files/poketool/trainer/trainers.json</t>
         </is>
       </c>
+      <c r="N139" s="2" t="inlineStr">
+        <is>
+          <t>후속 구현</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M139"/>
+  <autoFilter ref="A1:N139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Document and verify the v7 P1 boss effects rollout
</commit_message>
<xml_diff>
--- a/docs/boss-ace-tactics.xlsx
+++ b/docs/boss-ace-tactics.xlsx
@@ -663,7 +663,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -7935,7 +7935,7 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="N111" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9375,7 +9375,7 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="N130" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>v6 P0 적용</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v7 적용</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document and verify the v8 conditional boss and field effects
</commit_message>
<xml_diff>
--- a/docs/boss-ace-tactics.xlsx
+++ b/docs/boss-ace-tactics.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6927,7 +6927,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7359,7 +7359,7 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7791,7 +7791,7 @@
       </c>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -7935,7 +7935,7 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8007,7 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8223,7 +8223,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="N109" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="N110" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="N111" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="N113" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="N122" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9375,7 +9375,7 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="N126" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="N130" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>v7 적용</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -10239,7 +10239,7 @@
       </c>
       <c r="N136" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="N137" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="N139" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v8 적용</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document complete v9 boss moves and defer native checks for one batch
</commit_message>
<xml_diff>
--- a/docs/boss-ace-tactics.xlsx
+++ b/docs/boss-ace-tactics.xlsx
@@ -504,7 +504,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>현재 Lv100 전술(미변경)</t>
+          <t>v5 명세 당시 Lv100 전술</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
       </c>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2175,7 @@
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,7 @@
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3471,7 @@
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3903,7 +3903,7 @@
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="N52" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="N56" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
       </c>
       <c r="N57" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="N58" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="N59" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4767,7 +4767,7 @@
       </c>
       <c r="N60" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="N61" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="N62" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="N63" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="N64" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="N65" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5199,7 +5199,7 @@
       </c>
       <c r="N66" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="N67" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="N68" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5415,7 +5415,7 @@
       </c>
       <c r="N69" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="N70" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5631,7 +5631,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5847,7 +5847,7 @@
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6927,7 +6927,7 @@
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7143,7 @@
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7359,7 +7359,7 @@
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7503,7 @@
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7575,7 +7575,7 @@
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="N100" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="N101" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7791,7 +7791,7 @@
       </c>
       <c r="N102" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="N103" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -7935,7 +7935,7 @@
       </c>
       <c r="N104" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8007,7 +8007,7 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="N107" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8223,7 +8223,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="N109" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8367,7 @@
       </c>
       <c r="N110" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="N111" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
       </c>
       <c r="N112" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8583,7 +8583,7 @@
       </c>
       <c r="N113" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8655,7 +8655,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8727,7 +8727,7 @@
       </c>
       <c r="N115" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="N116" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8871,7 +8871,7 @@
       </c>
       <c r="N117" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -8943,7 +8943,7 @@
       </c>
       <c r="N118" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9015,7 +9015,7 @@
       </c>
       <c r="N119" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9087,7 +9087,7 @@
       </c>
       <c r="N120" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="N121" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9231,7 +9231,7 @@
       </c>
       <c r="N122" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9303,7 +9303,7 @@
       </c>
       <c r="N123" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9375,7 +9375,7 @@
       </c>
       <c r="N124" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9447,7 @@
       </c>
       <c r="N125" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9519,7 +9519,7 @@
       </c>
       <c r="N126" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       </c>
       <c r="N127" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9663,7 +9663,7 @@
       </c>
       <c r="N128" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9735,7 +9735,7 @@
       </c>
       <c r="N129" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9807,7 +9807,7 @@
       </c>
       <c r="N130" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="N131" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -9951,7 +9951,7 @@
       </c>
       <c r="N132" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="N133" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10095,7 +10095,7 @@
       </c>
       <c r="N134" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="N135" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10239,7 +10239,7 @@
       </c>
       <c r="N136" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10311,7 +10311,7 @@
       </c>
       <c r="N137" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10383,7 +10383,7 @@
       </c>
       <c r="N138" s="2" t="inlineStr">
         <is>
-          <t>후속 구현</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>
@@ -10455,7 +10455,7 @@
       </c>
       <c r="N139" s="2" t="inlineStr">
         <is>
-          <t>v8 적용</t>
+          <t>v9 적용</t>
         </is>
       </c>
     </row>

</xml_diff>